<commit_message>
feat: dar mayor peso al patron en entrenamiento y prediccion
</commit_message>
<xml_diff>
--- a/Produccion Astroflores BL25-26-27-28 a la Semana 18_entrenamiento.xlsx
+++ b/Produccion Astroflores BL25-26-27-28 a la Semana 18_entrenamiento.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="0" windowWidth="8565" windowHeight="11640"/>
+    <workbookView xWindow="-120" yWindow="0" windowWidth="9435" windowHeight="11640"/>
   </bookViews>
   <sheets>
     <sheet name="Astroflores" sheetId="1" r:id="rId1"/>
@@ -219,7 +219,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -250,6 +250,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -579,7 +582,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -602,10 +605,10 @@
     <col min="9" max="9" width="14" style="2" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="13.125" style="2" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="14.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.125" style="2" hidden="1" customWidth="1"/>
     <col min="13" max="15" width="7.875" style="2" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="8.625" style="2" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="8.625" style="2" customWidth="1"/>
+    <col min="17" max="17" width="12.25" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="16384" width="11.375" style="2"/>
   </cols>
   <sheetData>
@@ -5072,11 +5075,11 @@
         <v>1.7773726785917738</v>
       </c>
       <c r="R72" s="24">
-        <v>4292</v>
+        <v>5743</v>
       </c>
       <c r="S72" s="13">
         <f t="shared" si="5"/>
-        <v>0.15345167652859962</v>
+        <v>-0.13274161735700196</v>
       </c>
     </row>
     <row r="73" spans="1:20" hidden="1">
@@ -5103,7 +5106,7 @@
         <v>028COTOPAXI</v>
       </c>
       <c r="H73" s="23">
-        <v>9000</v>
+        <v>6000</v>
       </c>
       <c r="I73" s="3">
         <v>8505</v>
@@ -5131,14 +5134,14 @@
       </c>
       <c r="Q73" s="16">
         <f t="shared" si="4"/>
-        <v>3.1550994294528532</v>
+        <v>2.1033996196352356</v>
       </c>
       <c r="R73" s="24">
-        <v>7473</v>
+        <v>7652</v>
       </c>
       <c r="S73" s="12">
         <f t="shared" si="5"/>
-        <v>0.16966666666666666</v>
+        <v>-0.27533333333333332</v>
       </c>
     </row>
     <row r="74" spans="1:20" hidden="1">
@@ -5165,7 +5168,7 @@
         <v>028COTOPAXI</v>
       </c>
       <c r="H74" s="23">
-        <v>8250</v>
+        <v>6450</v>
       </c>
       <c r="I74" s="3">
         <v>8421</v>
@@ -5193,14 +5196,14 @@
       </c>
       <c r="Q74" s="16">
         <f t="shared" si="4"/>
-        <v>2.8921744769984485</v>
+        <v>2.2611545911078781</v>
       </c>
       <c r="R74" s="24">
-        <v>8101</v>
+        <v>5625</v>
       </c>
       <c r="S74" s="12">
         <f t="shared" si="5"/>
-        <v>1.8060606060606062E-2</v>
+        <v>0.12790697674418605</v>
       </c>
     </row>
     <row r="75" spans="1:20" hidden="1">
@@ -5258,14 +5261,14 @@
         <v>2.4714945530714014</v>
       </c>
       <c r="R75" s="24">
-        <v>7757</v>
+        <v>6604</v>
       </c>
       <c r="S75" s="12">
         <f t="shared" si="5"/>
-        <v>-0.10028368794326241</v>
-      </c>
-    </row>
-    <row r="76" spans="1:20" hidden="1">
+        <v>6.3262411347517727E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20">
       <c r="A76" s="9">
         <v>2025</v>
       </c>
@@ -5327,7 +5330,7 @@
         <v>3.0877107403802166E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:20" hidden="1">
+    <row r="77" spans="1:20">
       <c r="A77" s="9">
         <v>2025</v>
       </c>
@@ -5389,7 +5392,7 @@
         <v>0.48232224000061391</v>
       </c>
     </row>
-    <row r="78" spans="1:20" hidden="1">
+    <row r="78" spans="1:20">
       <c r="A78" s="9">
         <v>2025</v>
       </c>
@@ -5451,7 +5454,7 @@
         <v>7.1741781400531304E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:20" hidden="1">
+    <row r="79" spans="1:20">
       <c r="A79" s="9">
         <v>2025</v>
       </c>
@@ -5513,7 +5516,7 @@
         <v>0.71613773256725466</v>
       </c>
     </row>
-    <row r="80" spans="1:20" hidden="1">
+    <row r="80" spans="1:20">
       <c r="A80" s="9">
         <v>2025</v>
       </c>
@@ -5575,7 +5578,7 @@
         <v>0.19486637393481399</v>
       </c>
     </row>
-    <row r="81" spans="1:19" hidden="1">
+    <row r="81" spans="1:19">
       <c r="A81" s="9">
         <v>2025</v>
       </c>
@@ -5637,7 +5640,7 @@
         <v>0.15220497936786434</v>
       </c>
     </row>
-    <row r="82" spans="1:19" hidden="1">
+    <row r="82" spans="1:19">
       <c r="A82" s="9">
         <v>2025</v>
       </c>
@@ -5699,7 +5702,7 @@
         <v>-6.9756440217103671E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:19" hidden="1">
+    <row r="83" spans="1:19">
       <c r="A83" s="9">
         <v>2025</v>
       </c>
@@ -5761,7 +5764,7 @@
         <v>-1.4489413568261432E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:19" hidden="1">
+    <row r="84" spans="1:19">
       <c r="A84" s="9">
         <v>2025</v>
       </c>
@@ -5823,7 +5826,7 @@
         <v>-5.8557406002925638E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:19" hidden="1">
+    <row r="85" spans="1:19">
       <c r="A85" s="9">
         <v>2025</v>
       </c>
@@ -5885,7 +5888,7 @@
         <v>-7.3540277409036514E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:19" hidden="1">
+    <row r="86" spans="1:19">
       <c r="A86" s="9">
         <v>2025</v>
       </c>
@@ -5947,7 +5950,7 @@
         <v>-8.2905192402472683E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:19" hidden="1">
+    <row r="87" spans="1:19">
       <c r="A87" s="9">
         <v>2025</v>
       </c>
@@ -6009,7 +6012,7 @@
         <v>-5.1895408620424653E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:19" hidden="1">
+    <row r="88" spans="1:19">
       <c r="A88" s="9">
         <v>2025</v>
       </c>
@@ -6071,7 +6074,7 @@
         <v>-5.6672425162644868E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:19" hidden="1">
+    <row r="89" spans="1:19">
       <c r="A89" s="9">
         <v>2025</v>
       </c>
@@ -6133,7 +6136,7 @@
         <v>-6.1072421819018723E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:19" hidden="1">
+    <row r="90" spans="1:19">
       <c r="A90" s="9">
         <v>2025</v>
       </c>
@@ -6195,7 +6198,7 @@
         <v>-1.8665685401199984E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:19" hidden="1">
+    <row r="91" spans="1:19">
       <c r="A91" s="9">
         <v>2025</v>
       </c>
@@ -6257,7 +6260,7 @@
         <v>-0.1109071086567797</v>
       </c>
     </row>
-    <row r="92" spans="1:19" hidden="1">
+    <row r="92" spans="1:19">
       <c r="A92" s="9">
         <v>2025</v>
       </c>
@@ -6319,7 +6322,7 @@
         <v>3.6813856283518763E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:19" hidden="1">
+    <row r="93" spans="1:19">
       <c r="A93" s="9">
         <v>2025</v>
       </c>
@@ -6381,7 +6384,7 @@
         <v>0.37417401418841234</v>
       </c>
     </row>
-    <row r="94" spans="1:19" hidden="1">
+    <row r="94" spans="1:19">
       <c r="A94" s="9">
         <v>2025</v>
       </c>
@@ -6443,7 +6446,7 @@
         <v>-0.10727216710705835</v>
       </c>
     </row>
-    <row r="95" spans="1:19" hidden="1">
+    <row r="95" spans="1:19">
       <c r="A95" s="9">
         <v>2025</v>
       </c>
@@ -6505,7 +6508,7 @@
         <v>-0.11636462174515899</v>
       </c>
     </row>
-    <row r="96" spans="1:19" hidden="1">
+    <row r="96" spans="1:19">
       <c r="A96" s="9">
         <v>2025</v>
       </c>
@@ -6567,7 +6570,7 @@
         <v>-3.1679885994972505E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:19" hidden="1">
+    <row r="97" spans="1:19">
       <c r="A97" s="9">
         <v>2025</v>
       </c>
@@ -6629,7 +6632,7 @@
         <v>-6.7292410778161837E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:19" hidden="1">
+    <row r="98" spans="1:19">
       <c r="A98" s="9">
         <v>2025</v>
       </c>
@@ -6691,7 +6694,7 @@
         <v>-7.9848657285039246E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:19" hidden="1">
+    <row r="99" spans="1:19">
       <c r="A99" s="9">
         <v>2025</v>
       </c>
@@ -6753,7 +6756,7 @@
         <v>-7.9141357373170393E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:19" hidden="1">
+    <row r="100" spans="1:19">
       <c r="A100" s="9">
         <v>2025</v>
       </c>
@@ -6815,7 +6818,7 @@
         <v>-0.27108548052540982</v>
       </c>
     </row>
-    <row r="101" spans="1:19" hidden="1">
+    <row r="101" spans="1:19">
       <c r="A101" s="9">
         <v>2025</v>
       </c>
@@ -6877,7 +6880,7 @@
         <v>-8.5799642160727718E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:19" hidden="1">
+    <row r="102" spans="1:19">
       <c r="A102" s="9">
         <v>2025</v>
       </c>
@@ -6939,7 +6942,7 @@
         <v>-6.7524196120803903E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:19" hidden="1">
+    <row r="103" spans="1:19">
       <c r="A103" s="9">
         <v>2025</v>
       </c>
@@ -7001,7 +7004,7 @@
         <v>-8.0830364883254346E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:19" hidden="1">
+    <row r="104" spans="1:19">
       <c r="A104" s="9">
         <v>2025</v>
       </c>
@@ -7063,7 +7066,7 @@
         <v>-7.8173930524943314E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:19" hidden="1">
+    <row r="105" spans="1:19">
       <c r="A105" s="9">
         <v>2025</v>
       </c>
@@ -7125,7 +7128,7 @@
         <v>-6.8749726539840669E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:19" hidden="1">
+    <row r="106" spans="1:19">
       <c r="A106" s="9">
         <v>2025</v>
       </c>
@@ -7187,7 +7190,7 @@
         <v>-0.10547516270322926</v>
       </c>
     </row>
-    <row r="107" spans="1:19" hidden="1">
+    <row r="107" spans="1:19">
       <c r="A107" s="9">
         <v>2025</v>
       </c>
@@ -7249,7 +7252,7 @@
         <v>-7.5689962185422593E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:19" hidden="1">
+    <row r="108" spans="1:19">
       <c r="A108" s="9">
         <v>2025</v>
       </c>
@@ -7311,7 +7314,7 @@
         <v>-8.6860450120132229E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:19" hidden="1">
+    <row r="109" spans="1:19">
       <c r="A109" s="9">
         <v>2025</v>
       </c>
@@ -7373,7 +7376,7 @@
         <v>-7.9570005258245341E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:19" hidden="1">
+    <row r="110" spans="1:19">
       <c r="A110" s="9">
         <v>2025</v>
       </c>
@@ -7435,7 +7438,7 @@
         <v>-8.0573115337078866E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:19" hidden="1">
+    <row r="111" spans="1:19">
       <c r="A111" s="9">
         <v>2025</v>
       </c>
@@ -7497,7 +7500,7 @@
         <v>-6.3323662105379236E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:19" hidden="1">
+    <row r="112" spans="1:19">
       <c r="A112" s="9">
         <v>2025</v>
       </c>
@@ -7559,7 +7562,7 @@
         <v>-4.7619016080628011E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:19" hidden="1">
+    <row r="113" spans="1:19">
       <c r="A113" s="9">
         <v>2025</v>
       </c>
@@ -7621,7 +7624,7 @@
         <v>-8.3091857636765534E-2</v>
       </c>
     </row>
-    <row r="114" spans="1:19" hidden="1">
+    <row r="114" spans="1:19">
       <c r="A114" s="9">
         <v>2025</v>
       </c>
@@ -7683,7 +7686,7 @@
         <v>-7.4082609984534184E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:19" hidden="1">
+    <row r="115" spans="1:19">
       <c r="A115" s="9">
         <v>2025</v>
       </c>
@@ -7745,7 +7748,7 @@
         <v>-6.9359868488869797E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:19" hidden="1">
+    <row r="116" spans="1:19">
       <c r="A116" s="9">
         <v>2025</v>
       </c>
@@ -7807,7 +7810,7 @@
         <v>-6.1659699138490426E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:19" hidden="1">
+    <row r="117" spans="1:19">
       <c r="A117" s="9">
         <v>2025</v>
       </c>
@@ -7869,7 +7872,7 @@
         <v>-7.2671138117027662E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:19" hidden="1">
+    <row r="118" spans="1:19">
       <c r="A118" s="9">
         <v>2025</v>
       </c>
@@ -7931,7 +7934,7 @@
         <v>-7.6463298222950532E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:19" hidden="1">
+    <row r="119" spans="1:19">
       <c r="A119" s="9">
         <v>2025</v>
       </c>
@@ -7993,7 +7996,7 @@
         <v>-7.4840069348663746E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:19" hidden="1">
+    <row r="120" spans="1:19">
       <c r="A120" s="9">
         <v>2025</v>
       </c>
@@ -8055,7 +8058,7 @@
         <v>-7.3013019409203614E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:19" hidden="1">
+    <row r="121" spans="1:19">
       <c r="A121" s="9">
         <v>2025</v>
       </c>
@@ -8117,7 +8120,7 @@
         <v>-7.0874528774256901E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:19" hidden="1">
+    <row r="122" spans="1:19">
       <c r="A122" s="9">
         <v>2025</v>
       </c>
@@ -8179,7 +8182,7 @@
         <v>-8.4059952221872458E-2</v>
       </c>
     </row>
-    <row r="123" spans="1:19" hidden="1">
+    <row r="123" spans="1:19">
       <c r="A123" s="9">
         <v>2025</v>
       </c>
@@ -8241,7 +8244,7 @@
         <v>-6.4388680010805291E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:19" hidden="1">
+    <row r="124" spans="1:19">
       <c r="A124" s="9">
         <v>2025</v>
       </c>
@@ -8303,7 +8306,7 @@
         <v>-7.8627350883919048E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:19" hidden="1">
+    <row r="125" spans="1:19">
       <c r="A125" s="9">
         <v>2025</v>
       </c>
@@ -8365,7 +8368,7 @@
         <v>-7.2573043883947308E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:19" hidden="1">
+    <row r="126" spans="1:19">
       <c r="A126" s="9">
         <v>2025</v>
       </c>
@@ -8427,7 +8430,7 @@
         <v>-7.6994438849656177E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:19" hidden="1">
+    <row r="127" spans="1:19">
       <c r="A127" s="9">
         <v>2025</v>
       </c>
@@ -8489,7 +8492,7 @@
         <v>-8.1224905439873846E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:19" hidden="1">
+    <row r="128" spans="1:19">
       <c r="A128" s="9">
         <v>2026</v>
       </c>
@@ -8551,7 +8554,7 @@
         <v>-7.416234007518023E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:20" hidden="1">
+    <row r="129" spans="1:20">
       <c r="A129" s="9">
         <v>2026</v>
       </c>
@@ -8613,7 +8616,7 @@
         <v>-9.2878631357780864E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:20" hidden="1">
+    <row r="130" spans="1:20">
       <c r="A130" s="9">
         <v>2026</v>
       </c>
@@ -8675,7 +8678,7 @@
         <v>-9.4707097853609729E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:20" hidden="1">
+    <row r="131" spans="1:20">
       <c r="A131" s="9">
         <v>2026</v>
       </c>
@@ -8737,7 +8740,7 @@
         <v>2.4654747366117903E-3</v>
       </c>
     </row>
-    <row r="132" spans="1:20" hidden="1">
+    <row r="132" spans="1:20">
       <c r="A132" s="9">
         <v>2026</v>
       </c>
@@ -8799,7 +8802,7 @@
         <v>8.8858666501388434E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:20" hidden="1">
+    <row r="133" spans="1:20">
       <c r="A133" s="9">
         <v>2026</v>
       </c>
@@ -8861,7 +8864,7 @@
         <v>-8.46938833293404E-2</v>
       </c>
     </row>
-    <row r="134" spans="1:20" hidden="1">
+    <row r="134" spans="1:20">
       <c r="A134" s="9">
         <v>2026</v>
       </c>
@@ -8923,7 +8926,7 @@
         <v>-7.1763804180799626E-2</v>
       </c>
     </row>
-    <row r="135" spans="1:20" hidden="1">
+    <row r="135" spans="1:20">
       <c r="A135" s="9">
         <v>2026</v>
       </c>
@@ -8985,7 +8988,7 @@
         <v>-0.14493088259243034</v>
       </c>
     </row>
-    <row r="136" spans="1:20" hidden="1">
+    <row r="136" spans="1:20">
       <c r="A136" s="9">
         <v>2026</v>
       </c>
@@ -9047,7 +9050,7 @@
         <v>-0.10179525183474719</v>
       </c>
     </row>
-    <row r="137" spans="1:20" hidden="1">
+    <row r="137" spans="1:20">
       <c r="A137" s="9">
         <v>2026</v>
       </c>
@@ -9109,7 +9112,7 @@
         <v>-0.10631680117039559</v>
       </c>
     </row>
-    <row r="138" spans="1:20" hidden="1">
+    <row r="138" spans="1:20">
       <c r="A138" s="9">
         <v>2026</v>
       </c>
@@ -9171,7 +9174,7 @@
         <v>-7.789343096575857E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:20" hidden="1">
+    <row r="139" spans="1:20">
       <c r="A139" s="9">
         <v>2026</v>
       </c>
@@ -9233,7 +9236,7 @@
         <v>0.38560074434951769</v>
       </c>
     </row>
-    <row r="140" spans="1:20" hidden="1">
+    <row r="140" spans="1:20">
       <c r="A140" s="9">
         <v>2026</v>
       </c>
@@ -9295,7 +9298,7 @@
         <v>-6.1684520755901827E-2</v>
       </c>
     </row>
-    <row r="141" spans="1:20" hidden="1">
+    <row r="141" spans="1:20">
       <c r="A141" s="9">
         <v>2026</v>
       </c>
@@ -9357,7 +9360,7 @@
         <v>-8.2554854016739301E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:20" hidden="1">
+    <row r="142" spans="1:20">
       <c r="A142" s="9">
         <v>2026</v>
       </c>
@@ -9419,7 +9422,7 @@
         <v>-0.12516835104958446</v>
       </c>
     </row>
-    <row r="143" spans="1:20" hidden="1">
+    <row r="143" spans="1:20">
       <c r="A143" s="9">
         <v>2026</v>
       </c>
@@ -9484,7 +9487,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:20" hidden="1">
+    <row r="144" spans="1:20">
       <c r="A144" s="9">
         <v>2026</v>
       </c>
@@ -9549,7 +9552,7 @@
         <v>0.69</v>
       </c>
     </row>
-    <row r="145" spans="1:20" hidden="1">
+    <row r="145" spans="1:20">
       <c r="A145" s="9">
         <v>2026</v>
       </c>
@@ -9614,7 +9617,7 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="146" spans="1:20" hidden="1">
+    <row r="146" spans="1:20">
       <c r="A146" s="9">
         <v>2026</v>
       </c>
@@ -9669,14 +9672,14 @@
         <v>2.7764874979185108</v>
       </c>
       <c r="R146" s="24">
-        <v>8965</v>
+        <v>8085</v>
       </c>
       <c r="S146" s="13">
         <f t="shared" si="8"/>
-        <v>-0.13194444444444445</v>
-      </c>
-    </row>
-    <row r="147" spans="1:20" hidden="1">
+        <v>-2.0833333333333332E-2</v>
+      </c>
+    </row>
+    <row r="147" spans="1:20">
       <c r="A147" s="9">
         <v>2026</v>
       </c>
@@ -9700,7 +9703,7 @@
         <v>028DEEP PURPLE</v>
       </c>
       <c r="H147" s="23">
-        <v>11700</v>
+        <v>6660</v>
       </c>
       <c r="I147" s="3">
         <v>7586</v>
@@ -9728,17 +9731,17 @@
       </c>
       <c r="Q147" s="16">
         <f t="shared" si="7"/>
-        <v>4.1016292582887086</v>
+        <v>2.3347735777951111</v>
       </c>
       <c r="R147" s="24">
-        <v>13524</v>
+        <v>8173</v>
       </c>
       <c r="S147" s="12">
         <f t="shared" si="8"/>
-        <v>-0.1558974358974359</v>
-      </c>
-    </row>
-    <row r="148" spans="1:20" hidden="1">
+        <v>-0.22717717717717717</v>
+      </c>
+    </row>
+    <row r="148" spans="1:20">
       <c r="A148" s="9">
         <v>2026</v>
       </c>
@@ -9762,7 +9765,7 @@
         <v>028DEEP PURPLE</v>
       </c>
       <c r="H148" s="23">
-        <v>5580</v>
+        <v>6270</v>
       </c>
       <c r="I148" s="3">
         <v>6393</v>
@@ -9790,17 +9793,17 @@
       </c>
       <c r="Q148" s="16">
         <f t="shared" si="7"/>
-        <v>1.9561616462607689</v>
+        <v>2.1980526025188212</v>
       </c>
       <c r="R148" s="24">
-        <v>5855</v>
+        <v>8405</v>
       </c>
       <c r="S148" s="12">
         <f t="shared" si="8"/>
-        <v>-4.9283154121863799E-2</v>
-      </c>
-    </row>
-    <row r="149" spans="1:20" hidden="1">
+        <v>-0.34051036682615632</v>
+      </c>
+    </row>
+    <row r="149" spans="1:20">
       <c r="A149" s="9">
         <v>2026</v>
       </c>
@@ -9855,11 +9858,11 @@
         <v>1.609100709020955</v>
       </c>
       <c r="R149" s="24">
-        <v>4969</v>
+        <v>8160</v>
       </c>
       <c r="S149" s="12">
         <f t="shared" si="8"/>
-        <v>-8.2570806100217858E-2</v>
+        <v>-0.77777777777777779</v>
       </c>
     </row>
     <row r="150" spans="1:20" hidden="1">
@@ -14266,11 +14269,11 @@
         <v>2.8711404808020964</v>
       </c>
       <c r="R220" s="24">
-        <v>3636</v>
+        <v>4310</v>
       </c>
       <c r="S220" s="13">
         <f>+(H220-R220)/H220</f>
-        <v>-0.15428571428571428</v>
+        <v>-0.36825396825396828</v>
       </c>
     </row>
     <row r="221" spans="1:20" hidden="1">
@@ -14297,7 +14300,7 @@
         <v>026LOLA</v>
       </c>
       <c r="H221" s="23">
-        <v>4280</v>
+        <v>3075</v>
       </c>
       <c r="I221" s="3">
         <v>4263</v>
@@ -14325,14 +14328,14 @@
       </c>
       <c r="Q221" s="16">
         <f t="shared" si="10"/>
-        <v>3.9011051612168166</v>
+        <v>2.8027799931639512</v>
       </c>
       <c r="R221" s="24">
-        <v>4986</v>
+        <v>3800</v>
       </c>
       <c r="S221" s="12">
         <f t="shared" si="11"/>
-        <v>-0.16495327102803739</v>
+        <v>-0.23577235772357724</v>
       </c>
     </row>
     <row r="222" spans="1:20" hidden="1">
@@ -14359,7 +14362,7 @@
         <v>026LOLA</v>
       </c>
       <c r="H222" s="23">
-        <v>3420</v>
+        <v>5800</v>
       </c>
       <c r="I222" s="3">
         <v>4590</v>
@@ -14387,14 +14390,14 @@
       </c>
       <c r="Q222" s="16">
         <f t="shared" si="10"/>
-        <v>3.1172382362994191</v>
+        <v>5.2865443773498919</v>
       </c>
       <c r="R222" s="24">
-        <v>3938</v>
+        <v>4738</v>
       </c>
       <c r="S222" s="12">
         <f t="shared" si="11"/>
-        <v>-0.15146198830409358</v>
+        <v>0.18310344827586206</v>
       </c>
     </row>
     <row r="223" spans="1:20" hidden="1">
@@ -14452,11 +14455,11 @@
         <v>4.4297595989518062</v>
       </c>
       <c r="R223" s="24">
-        <v>5812</v>
+        <v>3924</v>
       </c>
       <c r="S223" s="12">
         <f t="shared" si="11"/>
-        <v>-0.19588477366255144</v>
+        <v>0.19259259259259259</v>
       </c>
     </row>
     <row r="224" spans="1:20" hidden="1">
@@ -18760,7 +18763,7 @@
         <f t="shared" si="12"/>
         <v>026PALOMA</v>
       </c>
-      <c r="H293" s="24">
+      <c r="H293" s="26">
         <v>10703</v>
       </c>
       <c r="I293" s="6">
@@ -18823,7 +18826,7 @@
         <v>026PALOMA</v>
       </c>
       <c r="H294" s="24">
-        <v>5698</v>
+        <v>4200</v>
       </c>
       <c r="I294" s="3">
         <v>9396</v>
@@ -18851,14 +18854,14 @@
       </c>
       <c r="Q294" s="16">
         <f t="shared" si="13"/>
-        <v>1.9975285054469285</v>
+        <v>1.4723797337446647</v>
       </c>
       <c r="R294" s="24">
-        <v>6745</v>
+        <v>6443</v>
       </c>
       <c r="S294" s="12">
         <f t="shared" si="14"/>
-        <v>-0.18374868374868375</v>
+        <v>-0.53404761904761899</v>
       </c>
     </row>
     <row r="295" spans="1:19" hidden="1">
@@ -18885,7 +18888,7 @@
         <v>026PALOMA</v>
       </c>
       <c r="H295" s="25">
-        <v>7982</v>
+        <v>4125</v>
       </c>
       <c r="I295" s="3">
         <v>6201</v>
@@ -18913,14 +18916,14 @@
       </c>
       <c r="Q295" s="16">
         <f t="shared" si="13"/>
-        <v>2.7982226273214081</v>
+        <v>1.4460872384992243</v>
       </c>
       <c r="R295" s="24">
-        <v>9011</v>
+        <v>6785</v>
       </c>
       <c r="S295" s="12">
         <f t="shared" si="14"/>
-        <v>-0.12891505888248558</v>
+        <v>-0.64484848484848489</v>
       </c>
     </row>
     <row r="296" spans="1:19" hidden="1">
@@ -18947,7 +18950,7 @@
         <v>026PALOMA</v>
       </c>
       <c r="H296" s="25">
-        <v>5249</v>
+        <v>6600</v>
       </c>
       <c r="I296" s="3">
         <v>6489</v>
@@ -18975,14 +18978,14 @@
       </c>
       <c r="Q296" s="16">
         <f t="shared" si="13"/>
-        <v>1.8401241005775584</v>
+        <v>2.3137395815987589</v>
       </c>
       <c r="R296" s="24">
-        <v>5652</v>
+        <v>5624</v>
       </c>
       <c r="S296" s="12">
         <f t="shared" si="14"/>
-        <v>-7.6776528862640497E-2</v>
+        <v>0.14787878787878789</v>
       </c>
     </row>
     <row r="297" spans="1:19" hidden="1">
@@ -19040,11 +19043,11 @@
         <v>1.7317990201663438</v>
       </c>
       <c r="R297" s="24">
-        <v>5260</v>
+        <v>5499</v>
       </c>
       <c r="S297" s="12">
         <f t="shared" si="14"/>
-        <v>-6.4777327935222673E-2</v>
+        <v>-0.11315789473684211</v>
       </c>
     </row>
     <row r="298" spans="1:19" hidden="1">
@@ -23482,7 +23485,7 @@
         <v>025PINK MONDIAL</v>
       </c>
       <c r="H369" s="23">
-        <v>7575</v>
+        <v>6025</v>
       </c>
       <c r="I369" s="3">
         <v>7114</v>
@@ -23510,14 +23513,14 @@
       </c>
       <c r="Q369" s="16">
         <f t="shared" si="16"/>
-        <v>2.4658599954275795</v>
+        <v>1.961294583821936</v>
       </c>
       <c r="R369" s="24">
         <v>7821</v>
       </c>
       <c r="S369" s="12">
         <f t="shared" si="17"/>
-        <v>-3.2475247524752476E-2</v>
+        <v>-0.29809128630705395</v>
       </c>
     </row>
     <row r="370" spans="1:19" hidden="1">
@@ -23544,7 +23547,7 @@
         <v>025PINK MONDIAL</v>
       </c>
       <c r="H370" s="23">
-        <v>4350</v>
+        <v>5050</v>
       </c>
       <c r="I370" s="3">
         <v>7150</v>
@@ -23572,14 +23575,14 @@
       </c>
       <c r="Q370" s="16">
         <f t="shared" si="16"/>
-        <v>1.4160384132158377</v>
+        <v>1.6439066636183861</v>
       </c>
       <c r="R370" s="24">
         <v>4663</v>
       </c>
       <c r="S370" s="12">
         <f t="shared" si="17"/>
-        <v>-7.1954022988505742E-2</v>
+        <v>7.6633663366336632E-2</v>
       </c>
     </row>
     <row r="371" spans="1:19" hidden="1">
@@ -31661,7 +31664,7 @@
         <v>027SATISFACTION</v>
       </c>
       <c r="H508" s="3">
-        <v>5790</v>
+        <v>4440</v>
       </c>
       <c r="I508" s="3">
         <v>4410</v>
@@ -31689,14 +31692,14 @@
       </c>
       <c r="Q508" s="16">
         <f t="shared" si="22"/>
-        <v>2.1989290190270023</v>
+        <v>1.6862253617409138</v>
       </c>
       <c r="R508" s="24">
         <v>6562</v>
       </c>
       <c r="S508" s="11">
         <f t="shared" si="23"/>
-        <v>-0.13333333333333333</v>
+        <v>-0.47792792792792793</v>
       </c>
     </row>
     <row r="509" spans="1:20" hidden="1">
@@ -31723,7 +31726,7 @@
         <v>027SATISFACTION</v>
       </c>
       <c r="H509" s="3">
-        <v>4230</v>
+        <v>5640</v>
       </c>
       <c r="I509" s="3">
         <v>4527</v>
@@ -31751,14 +31754,14 @@
       </c>
       <c r="Q509" s="16">
         <f t="shared" si="22"/>
-        <v>1.6064714594964111</v>
+        <v>2.1419619459952148</v>
       </c>
       <c r="R509" s="24">
         <v>4694</v>
       </c>
       <c r="S509" s="11">
         <f t="shared" si="23"/>
-        <v>-0.10969267139479906</v>
+        <v>0.1677304964539007</v>
       </c>
     </row>
     <row r="510" spans="1:20" hidden="1">
@@ -31823,7 +31826,7 @@
         <v>-9.56989247311828E-2</v>
       </c>
     </row>
-    <row r="511" spans="1:20">
+    <row r="511" spans="1:20" hidden="1">
       <c r="A511" s="9">
         <v>2025</v>
       </c>
@@ -31885,7 +31888,7 @@
         <v>-5.443989868749901E-2</v>
       </c>
     </row>
-    <row r="512" spans="1:20">
+    <row r="512" spans="1:20" hidden="1">
       <c r="A512" s="9">
         <v>2025</v>
       </c>
@@ -31947,7 +31950,7 @@
         <v>0.33784748734962994</v>
       </c>
     </row>
-    <row r="513" spans="1:19">
+    <row r="513" spans="1:19" hidden="1">
       <c r="A513" s="9">
         <v>2025</v>
       </c>
@@ -32009,7 +32012,7 @@
         <v>-1.5746172400461576E-3</v>
       </c>
     </row>
-    <row r="514" spans="1:19">
+    <row r="514" spans="1:19" hidden="1">
       <c r="A514" s="9">
         <v>2025</v>
       </c>
@@ -32071,7 +32074,7 @@
         <v>0.64386016039643124</v>
       </c>
     </row>
-    <row r="515" spans="1:19">
+    <row r="515" spans="1:19" hidden="1">
       <c r="A515" s="9">
         <v>2025</v>
       </c>
@@ -32133,7 +32136,7 @@
         <v>0.25904988301186427</v>
       </c>
     </row>
-    <row r="516" spans="1:19">
+    <row r="516" spans="1:19" hidden="1">
       <c r="A516" s="9">
         <v>2025</v>
       </c>
@@ -32195,7 +32198,7 @@
         <v>0.24592833003101966</v>
       </c>
     </row>
-    <row r="517" spans="1:19">
+    <row r="517" spans="1:19" hidden="1">
       <c r="A517" s="9">
         <v>2025</v>
       </c>
@@ -32257,7 +32260,7 @@
         <v>-4.5944242148778153E-2</v>
       </c>
     </row>
-    <row r="518" spans="1:19">
+    <row r="518" spans="1:19" hidden="1">
       <c r="A518" s="9">
         <v>2025</v>
       </c>
@@ -32319,7 +32322,7 @@
         <v>-5.2661155278108815E-2</v>
       </c>
     </row>
-    <row r="519" spans="1:19">
+    <row r="519" spans="1:19" hidden="1">
       <c r="A519" s="9">
         <v>2025</v>
       </c>
@@ -32381,7 +32384,7 @@
         <v>-5.1872917704794359E-2</v>
       </c>
     </row>
-    <row r="520" spans="1:19">
+    <row r="520" spans="1:19" hidden="1">
       <c r="A520" s="9">
         <v>2025</v>
       </c>
@@ -32443,7 +32446,7 @@
         <v>-5.1789500404753143E-2</v>
       </c>
     </row>
-    <row r="521" spans="1:19">
+    <row r="521" spans="1:19" hidden="1">
       <c r="A521" s="9">
         <v>2025</v>
       </c>
@@ -32505,7 +32508,7 @@
         <v>-4.5822182773103619E-2</v>
       </c>
     </row>
-    <row r="522" spans="1:19">
+    <row r="522" spans="1:19" hidden="1">
       <c r="A522" s="9">
         <v>2025</v>
       </c>
@@ -32567,7 +32570,7 @@
         <v>8.305711321197376E-2</v>
       </c>
     </row>
-    <row r="523" spans="1:19">
+    <row r="523" spans="1:19" hidden="1">
       <c r="A523" s="9">
         <v>2025</v>
       </c>
@@ -32629,7 +32632,7 @@
         <v>-5.22651924359296E-2</v>
       </c>
     </row>
-    <row r="524" spans="1:19">
+    <row r="524" spans="1:19" hidden="1">
       <c r="A524" s="9">
         <v>2025</v>
       </c>
@@ -32691,7 +32694,7 @@
         <v>-5.6131399734409011E-2</v>
       </c>
     </row>
-    <row r="525" spans="1:19">
+    <row r="525" spans="1:19" hidden="1">
       <c r="A525" s="9">
         <v>2025</v>
       </c>
@@ -32753,7 +32756,7 @@
         <v>-7.3959179479694522E-3</v>
       </c>
     </row>
-    <row r="526" spans="1:19">
+    <row r="526" spans="1:19" hidden="1">
       <c r="A526" s="9">
         <v>2025</v>
       </c>
@@ -32815,7 +32818,7 @@
         <v>-3.4466167124361929E-2</v>
       </c>
     </row>
-    <row r="527" spans="1:19">
+    <row r="527" spans="1:19" hidden="1">
       <c r="A527" s="9">
         <v>2025</v>
       </c>
@@ -32877,7 +32880,7 @@
         <v>-4.1835256528830106E-2</v>
       </c>
     </row>
-    <row r="528" spans="1:19">
+    <row r="528" spans="1:19" hidden="1">
       <c r="A528" s="9">
         <v>2025</v>
       </c>
@@ -32939,7 +32942,7 @@
         <v>3.662111848627677E-2</v>
       </c>
     </row>
-    <row r="529" spans="1:19">
+    <row r="529" spans="1:19" hidden="1">
       <c r="A529" s="9">
         <v>2025</v>
       </c>
@@ -33001,7 +33004,7 @@
         <v>-4.9505006773268564E-2</v>
       </c>
     </row>
-    <row r="530" spans="1:19">
+    <row r="530" spans="1:19" hidden="1">
       <c r="A530" s="9">
         <v>2025</v>
       </c>
@@ -33063,7 +33066,7 @@
         <v>-4.8609350723670133E-2</v>
       </c>
     </row>
-    <row r="531" spans="1:19">
+    <row r="531" spans="1:19" hidden="1">
       <c r="A531" s="9">
         <v>2025</v>
       </c>
@@ -33125,7 +33128,7 @@
         <v>-6.3031623374298185E-2</v>
       </c>
     </row>
-    <row r="532" spans="1:19">
+    <row r="532" spans="1:19" hidden="1">
       <c r="A532" s="9">
         <v>2025</v>
       </c>
@@ -33187,7 +33190,7 @@
         <v>-6.6901230290556959E-2</v>
       </c>
     </row>
-    <row r="533" spans="1:19">
+    <row r="533" spans="1:19" hidden="1">
       <c r="A533" s="9">
         <v>2025</v>
       </c>
@@ -33249,7 +33252,7 @@
         <v>-5.0014290898666276E-2</v>
       </c>
     </row>
-    <row r="534" spans="1:19">
+    <row r="534" spans="1:19" hidden="1">
       <c r="A534" s="9">
         <v>2025</v>
       </c>
@@ -33311,7 +33314,7 @@
         <v>-5.6449581305727361E-3</v>
       </c>
     </row>
-    <row r="535" spans="1:19">
+    <row r="535" spans="1:19" hidden="1">
       <c r="A535" s="9">
         <v>2025</v>
       </c>
@@ -33373,7 +33376,7 @@
         <v>-2.1608208777733277E-2</v>
       </c>
     </row>
-    <row r="536" spans="1:19">
+    <row r="536" spans="1:19" hidden="1">
       <c r="A536" s="9">
         <v>2025</v>
       </c>
@@ -33435,7 +33438,7 @@
         <v>-5.1387112060961887E-2</v>
       </c>
     </row>
-    <row r="537" spans="1:19">
+    <row r="537" spans="1:19" hidden="1">
       <c r="A537" s="9">
         <v>2025</v>
       </c>
@@ -33497,7 +33500,7 @@
         <v>-0.15351170554471477</v>
       </c>
     </row>
-    <row r="538" spans="1:19">
+    <row r="538" spans="1:19" hidden="1">
       <c r="A538" s="9">
         <v>2025</v>
       </c>
@@ -33559,7 +33562,7 @@
         <v>-0.10481227707236242</v>
       </c>
     </row>
-    <row r="539" spans="1:19">
+    <row r="539" spans="1:19" hidden="1">
       <c r="A539" s="9">
         <v>2025</v>
       </c>
@@ -33621,7 +33624,7 @@
         <v>-4.9183063780923492E-2</v>
       </c>
     </row>
-    <row r="540" spans="1:19">
+    <row r="540" spans="1:19" hidden="1">
       <c r="A540" s="9">
         <v>2025</v>
       </c>
@@ -33683,7 +33686,7 @@
         <v>-1.3705568641491301E-2</v>
       </c>
     </row>
-    <row r="541" spans="1:19">
+    <row r="541" spans="1:19" hidden="1">
       <c r="A541" s="9">
         <v>2025</v>
       </c>
@@ -33745,7 +33748,7 @@
         <v>-7.6949530323245391E-2</v>
       </c>
     </row>
-    <row r="542" spans="1:19">
+    <row r="542" spans="1:19" hidden="1">
       <c r="A542" s="9">
         <v>2025</v>
       </c>
@@ -33807,7 +33810,7 @@
         <v>-5.0123304679888868E-2</v>
       </c>
     </row>
-    <row r="543" spans="1:19">
+    <row r="543" spans="1:19" hidden="1">
       <c r="A543" s="9">
         <v>2025</v>
       </c>
@@ -33869,7 +33872,7 @@
         <v>-5.2038452799273605E-2</v>
       </c>
     </row>
-    <row r="544" spans="1:19">
+    <row r="544" spans="1:19" hidden="1">
       <c r="A544" s="9">
         <v>2025</v>
       </c>
@@ -33931,7 +33934,7 @@
         <v>-6.0748700141355499E-2</v>
       </c>
     </row>
-    <row r="545" spans="1:19">
+    <row r="545" spans="1:19" hidden="1">
       <c r="A545" s="9">
         <v>2025</v>
       </c>
@@ -33993,7 +33996,7 @@
         <v>-9.0419919571597479E-2</v>
       </c>
     </row>
-    <row r="546" spans="1:19">
+    <row r="546" spans="1:19" hidden="1">
       <c r="A546" s="9">
         <v>2025</v>
       </c>
@@ -34055,7 +34058,7 @@
         <v>-5.0490650000137673E-2</v>
       </c>
     </row>
-    <row r="547" spans="1:19">
+    <row r="547" spans="1:19" hidden="1">
       <c r="A547" s="9">
         <v>2025</v>
       </c>
@@ -34117,7 +34120,7 @@
         <v>-5.2884591453338695E-2</v>
       </c>
     </row>
-    <row r="548" spans="1:19">
+    <row r="548" spans="1:19" hidden="1">
       <c r="A548" s="9">
         <v>2025</v>
       </c>
@@ -34179,7 +34182,7 @@
         <v>-5.5750963807099464E-2</v>
       </c>
     </row>
-    <row r="549" spans="1:19">
+    <row r="549" spans="1:19" hidden="1">
       <c r="A549" s="9">
         <v>2025</v>
       </c>
@@ -34241,7 +34244,7 @@
         <v>-8.1018341254971107E-2</v>
       </c>
     </row>
-    <row r="550" spans="1:19">
+    <row r="550" spans="1:19" hidden="1">
       <c r="A550" s="9">
         <v>2025</v>
       </c>
@@ -34303,7 +34306,7 @@
         <v>-6.4999232357152562E-2</v>
       </c>
     </row>
-    <row r="551" spans="1:19">
+    <row r="551" spans="1:19" hidden="1">
       <c r="A551" s="9">
         <v>2025</v>
       </c>
@@ -34365,7 +34368,7 @@
         <v>-5.0972968368580826E-2</v>
       </c>
     </row>
-    <row r="552" spans="1:19">
+    <row r="552" spans="1:19" hidden="1">
       <c r="A552" s="9">
         <v>2025</v>
       </c>
@@ -34427,7 +34430,7 @@
         <v>-4.2789815818707562E-2</v>
       </c>
     </row>
-    <row r="553" spans="1:19">
+    <row r="553" spans="1:19" hidden="1">
       <c r="A553" s="9">
         <v>2025</v>
       </c>
@@ -34489,7 +34492,7 @@
         <v>-4.2686431277672771E-2</v>
       </c>
     </row>
-    <row r="554" spans="1:19">
+    <row r="554" spans="1:19" hidden="1">
       <c r="A554" s="9">
         <v>2025</v>
       </c>
@@ -34551,7 +34554,7 @@
         <v>-5.7699220059668266E-2</v>
       </c>
     </row>
-    <row r="555" spans="1:19">
+    <row r="555" spans="1:19" hidden="1">
       <c r="A555" s="9">
         <v>2025</v>
       </c>
@@ -34613,7 +34616,7 @@
         <v>-5.4938523443591958E-2</v>
       </c>
     </row>
-    <row r="556" spans="1:19">
+    <row r="556" spans="1:19" hidden="1">
       <c r="A556" s="9">
         <v>2025</v>
       </c>
@@ -34675,7 +34678,7 @@
         <v>-5.936698219294817E-2</v>
       </c>
     </row>
-    <row r="557" spans="1:19">
+    <row r="557" spans="1:19" hidden="1">
       <c r="A557" s="9">
         <v>2025</v>
       </c>
@@ -34737,7 +34740,7 @@
         <v>-5.2174883797293063E-2</v>
       </c>
     </row>
-    <row r="558" spans="1:19">
+    <row r="558" spans="1:19" hidden="1">
       <c r="A558" s="9">
         <v>2025</v>
       </c>
@@ -34799,7 +34802,7 @@
         <v>-4.3948803149930625E-2</v>
       </c>
     </row>
-    <row r="559" spans="1:19">
+    <row r="559" spans="1:19" hidden="1">
       <c r="A559" s="9">
         <v>2025</v>
       </c>
@@ -34861,7 +34864,7 @@
         <v>-5.350877422497919E-2</v>
       </c>
     </row>
-    <row r="560" spans="1:19">
+    <row r="560" spans="1:19" hidden="1">
       <c r="A560" s="9">
         <v>2025</v>
       </c>
@@ -34923,7 +34926,7 @@
         <v>-5.8521381130006031E-2</v>
       </c>
     </row>
-    <row r="561" spans="1:19">
+    <row r="561" spans="1:19" hidden="1">
       <c r="A561" s="9">
         <v>2025</v>
       </c>
@@ -34974,7 +34977,7 @@
         <v>13.918303571428599</v>
       </c>
       <c r="Q561" s="16">
-        <f t="shared" si="25"/>
+        <f>+H561/K561</f>
         <v>1.6634385325281988</v>
       </c>
       <c r="R561" s="10">
@@ -34985,7 +34988,7 @@
         <v>-4.8385900450627295E-2</v>
       </c>
     </row>
-    <row r="562" spans="1:19">
+    <row r="562" spans="1:19" hidden="1">
       <c r="A562" s="9">
         <v>2025</v>
       </c>
@@ -35047,7 +35050,7 @@
         <v>-5.3963777527636682E-2</v>
       </c>
     </row>
-    <row r="563" spans="1:19">
+    <row r="563" spans="1:19" hidden="1">
       <c r="A563" s="9">
         <v>2026</v>
       </c>
@@ -35109,7 +35112,7 @@
         <v>-5.1412614095146476E-2</v>
       </c>
     </row>
-    <row r="564" spans="1:19">
+    <row r="564" spans="1:19" hidden="1">
       <c r="A564" s="9">
         <v>2026</v>
       </c>
@@ -35171,7 +35174,7 @@
         <v>-4.5284362774851684E-2</v>
       </c>
     </row>
-    <row r="565" spans="1:19">
+    <row r="565" spans="1:19" hidden="1">
       <c r="A565" s="9">
         <v>2026</v>
       </c>
@@ -35233,7 +35236,7 @@
         <v>-8.3885978751051921E-4</v>
       </c>
     </row>
-    <row r="566" spans="1:19">
+    <row r="566" spans="1:19" hidden="1">
       <c r="A566" s="9">
         <v>2026</v>
       </c>
@@ -35295,7 +35298,7 @@
         <v>-0.1329906146868938</v>
       </c>
     </row>
-    <row r="567" spans="1:19">
+    <row r="567" spans="1:19" hidden="1">
       <c r="A567" s="9">
         <v>2026</v>
       </c>
@@ -35357,7 +35360,7 @@
         <v>0.13372802127999847</v>
       </c>
     </row>
-    <row r="568" spans="1:19">
+    <row r="568" spans="1:19" hidden="1">
       <c r="A568" s="9">
         <v>2026</v>
       </c>
@@ -35419,7 +35422,7 @@
         <v>-7.2792191131655568E-2</v>
       </c>
     </row>
-    <row r="569" spans="1:19">
+    <row r="569" spans="1:19" hidden="1">
       <c r="A569" s="9">
         <v>2026</v>
       </c>
@@ -35481,7 +35484,7 @@
         <v>-0.18507766028257466</v>
       </c>
     </row>
-    <row r="570" spans="1:19">
+    <row r="570" spans="1:19" hidden="1">
       <c r="A570" s="9">
         <v>2026</v>
       </c>
@@ -35543,7 +35546,7 @@
         <v>-4.9879535952812797E-2</v>
       </c>
     </row>
-    <row r="571" spans="1:19">
+    <row r="571" spans="1:19" hidden="1">
       <c r="A571" s="9">
         <v>2026</v>
       </c>
@@ -35605,7 +35608,7 @@
         <v>-7.3746040147171801E-2</v>
       </c>
     </row>
-    <row r="572" spans="1:19">
+    <row r="572" spans="1:19" hidden="1">
       <c r="A572" s="9">
         <v>2026</v>
       </c>
@@ -35667,7 +35670,7 @@
         <v>-5.0337869380806761E-2</v>
       </c>
     </row>
-    <row r="573" spans="1:19">
+    <row r="573" spans="1:19" hidden="1">
       <c r="A573" s="9">
         <v>2026</v>
       </c>
@@ -35729,7 +35732,7 @@
         <v>-7.3657693591400217E-2</v>
       </c>
     </row>
-    <row r="574" spans="1:19">
+    <row r="574" spans="1:19" hidden="1">
       <c r="A574" s="9">
         <v>2026</v>
       </c>
@@ -35791,7 +35794,7 @@
         <v>-8.3885978751051921E-4</v>
       </c>
     </row>
-    <row r="575" spans="1:19">
+    <row r="575" spans="1:19" hidden="1">
       <c r="A575" s="9">
         <v>2026</v>
       </c>
@@ -35853,7 +35856,7 @@
         <v>-4.4439745611088377E-2</v>
       </c>
     </row>
-    <row r="576" spans="1:19">
+    <row r="576" spans="1:19" hidden="1">
       <c r="A576" s="9">
         <v>2026</v>
       </c>
@@ -35915,7 +35918,7 @@
         <v>-5.0522388411464746E-2</v>
       </c>
     </row>
-    <row r="577" spans="1:20">
+    <row r="577" spans="1:20" hidden="1">
       <c r="A577" s="9">
         <v>2026</v>
       </c>
@@ -35977,7 +35980,7 @@
         <v>-4.1207281509484446E-2</v>
       </c>
     </row>
-    <row r="578" spans="1:20">
+    <row r="578" spans="1:20" hidden="1">
       <c r="A578" s="9">
         <v>2026</v>
       </c>
@@ -36042,7 +36045,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="579" spans="1:20">
+    <row r="579" spans="1:20" hidden="1">
       <c r="A579" s="9">
         <v>2026</v>
       </c>
@@ -36107,7 +36110,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="580" spans="1:20">
+    <row r="580" spans="1:20" hidden="1">
       <c r="A580" s="9">
         <v>2026</v>
       </c>
@@ -36172,7 +36175,7 @@
         <v>0.92</v>
       </c>
     </row>
-    <row r="581" spans="1:20">
+    <row r="581" spans="1:20" hidden="1">
       <c r="A581" s="9">
         <v>2026</v>
       </c>
@@ -36227,14 +36230,14 @@
         <v>3.0192548706847444</v>
       </c>
       <c r="R581" s="24">
-        <v>6176</v>
+        <v>4743</v>
       </c>
       <c r="S581" s="13">
         <f t="shared" si="26"/>
-        <v>0.22314465408805031</v>
-      </c>
-    </row>
-    <row r="582" spans="1:20">
+        <v>0.40339622641509432</v>
+      </c>
+    </row>
+    <row r="582" spans="1:20" hidden="1">
       <c r="A582" s="9">
         <v>2026</v>
       </c>
@@ -36258,7 +36261,7 @@
         <v>027TIFFANY!</v>
       </c>
       <c r="H582" s="3">
-        <v>5520</v>
+        <v>5010</v>
       </c>
       <c r="I582" s="3">
         <v>4371</v>
@@ -36286,17 +36289,17 @@
       </c>
       <c r="Q582" s="16">
         <f t="shared" si="25"/>
-        <v>2.0963882875697846</v>
+        <v>1.9027002392617067</v>
       </c>
       <c r="R582" s="24">
-        <v>5983</v>
+        <v>5309</v>
       </c>
       <c r="S582" s="11">
         <f t="shared" si="26"/>
-        <v>-8.3876811594202905E-2</v>
-      </c>
-    </row>
-    <row r="583" spans="1:20">
+        <v>-5.9680638722554892E-2</v>
+      </c>
+    </row>
+    <row r="583" spans="1:20" hidden="1">
       <c r="A583" s="9">
         <v>2026</v>
       </c>
@@ -36320,7 +36323,7 @@
         <v>027TIFFANY!</v>
       </c>
       <c r="H583" s="3">
-        <v>4770</v>
+        <v>6420</v>
       </c>
       <c r="I583" s="3">
         <v>4623</v>
@@ -36348,17 +36351,17 @@
       </c>
       <c r="Q583" s="16">
         <f t="shared" si="25"/>
-        <v>1.8115529224108466</v>
+        <v>2.4381907257605104</v>
       </c>
       <c r="R583" s="24">
-        <v>5344</v>
+        <v>6022</v>
       </c>
       <c r="S583" s="11">
         <f t="shared" si="26"/>
-        <v>-0.12033542976939203</v>
-      </c>
-    </row>
-    <row r="584" spans="1:20">
+        <v>6.1993769470404983E-2</v>
+      </c>
+    </row>
+    <row r="584" spans="1:20" hidden="1">
       <c r="A584" s="9">
         <v>2026</v>
       </c>
@@ -36413,18 +36416,19 @@
         <v>1.6178648741027686</v>
       </c>
       <c r="R584" s="24">
-        <v>4600</v>
+        <v>5248</v>
       </c>
       <c r="S584" s="11">
         <f t="shared" si="26"/>
-        <v>-7.9812206572769953E-2</v>
+        <v>-0.23192488262910799</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S584">
+    <filterColumn colId="0"/>
     <filterColumn colId="5">
       <filters>
-        <filter val="TIFFANY!"/>
+        <filter val="DEEP PURPLE"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>